<commit_message>
Added Config.mat for better Code generation
</commit_message>
<xml_diff>
--- a/L1_Repo/ACC_Model/Testing/MIL/ACC_MIL.xlsx
+++ b/L1_Repo/ACC_Model/Testing/MIL/ACC_MIL.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="2999" uniqueCount="213">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="3466" uniqueCount="213">
   <si>
     <t>TimeRelative</t>
   </si>
@@ -27735,6 +27735,8 @@
       </c>
     </row>
     <row r="44" ht="15.75" customHeight="true">
+      <c r="A44" s="0"/>
+      <c r="B44" s="0"/>
       <c r="C44" s="0" t="s">
         <v>73</v>
       </c>

</xml_diff>